<commit_message>
2026-07-02 v2.2.0 - 7/1 작업분 체크포인트 (재고전망·과잉감축 개편, bom-sim/meeting/minutes 신규 화면, RAW 갱신)
</commit_message>
<xml_diff>
--- a/기초재고_재공품_RAW.xlsx
+++ b/기초재고_재공품_RAW.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1784" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1868" uniqueCount="357">
   <si>
     <t>회사코드</t>
   </si>
@@ -1037,6 +1037,51 @@
   </si>
   <si>
     <t>엔블로멧서방정0.3/1000mg(이나보글리플로진,메트포르민염산염)30T</t>
+  </si>
+  <si>
+    <t>1240</t>
+  </si>
+  <si>
+    <t>8400457</t>
+  </si>
+  <si>
+    <t>다이소 닥터베어 칼슘 마그네슘 비타민D 반제품</t>
+  </si>
+  <si>
+    <t>8400458</t>
+  </si>
+  <si>
+    <t>다이소 닥터베어 마그네슘 반제품</t>
+  </si>
+  <si>
+    <t>8400460</t>
+  </si>
+  <si>
+    <t>다이소 닥터베어 녹차카테킨 반제품</t>
+  </si>
+  <si>
+    <t>8400464</t>
+  </si>
+  <si>
+    <t>다이소 닥터베어 블랙마카 반제품</t>
+  </si>
+  <si>
+    <t>8400466</t>
+  </si>
+  <si>
+    <t>다이소 닥터베어 멀티비타민 미네랄 반제품</t>
+  </si>
+  <si>
+    <t>9401381</t>
+  </si>
+  <si>
+    <t>다이소 닥터베어 바나바잎 추출물 (30정)</t>
+  </si>
+  <si>
+    <t>9401669</t>
+  </si>
+  <si>
+    <t>Amway XS Essential 태국_6.4g*30(192g)</t>
   </si>
 </sst>
 </file>
@@ -1159,7 +1204,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1"/>
   </sheetPr>
-  <dimension ref="A1:R148"/>
+  <dimension ref="A1:R155"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" bestFit="1" width="5" customWidth="1"/>
@@ -9414,60 +9459,452 @@
         <v>15220328</v>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="J148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="K148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="L148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="M148" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="N148" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="O148" s="6">
+    <row r="148" outlineLevel="0" collapsed="0" hidden="0">
+      <c r="A148" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C148" s="3">
+        <v>5</v>
+      </c>
+      <c r="D148" s="3">
+        <v>5</v>
+      </c>
+      <c r="E148" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F148" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="G148" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="H148" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I148" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J148" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K148" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L148" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M148" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N148" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O148" s="3">
+        <v>0</v>
+      </c>
+      <c r="P148" s="3">
+        <v>53959945</v>
+      </c>
+      <c r="Q148" s="3">
+        <v>0</v>
+      </c>
+      <c r="R148" s="3">
+        <v>53959945</v>
+      </c>
+    </row>
+    <row r="149" outlineLevel="0" collapsed="0" hidden="0">
+      <c r="A149" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C149" s="3">
+        <v>5</v>
+      </c>
+      <c r="D149" s="3">
+        <v>5</v>
+      </c>
+      <c r="E149" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F149" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="G149" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="H149" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I149" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J149" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K149" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L149" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M149" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N149" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O149" s="3">
+        <v>0</v>
+      </c>
+      <c r="P149" s="3">
+        <v>51228454</v>
+      </c>
+      <c r="Q149" s="3">
+        <v>0</v>
+      </c>
+      <c r="R149" s="3">
+        <v>51228454</v>
+      </c>
+    </row>
+    <row r="150" outlineLevel="0" collapsed="0" hidden="0">
+      <c r="A150" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C150" s="3">
+        <v>5</v>
+      </c>
+      <c r="D150" s="3">
+        <v>5</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F150" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="G150" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="H150" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I150" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J150" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K150" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L150" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M150" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N150" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O150" s="3">
+        <v>0</v>
+      </c>
+      <c r="P150" s="3">
+        <v>97791556</v>
+      </c>
+      <c r="Q150" s="3">
+        <v>0</v>
+      </c>
+      <c r="R150" s="3">
+        <v>97791556</v>
+      </c>
+    </row>
+    <row r="151" outlineLevel="0" collapsed="0" hidden="0">
+      <c r="A151" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C151" s="3">
+        <v>5</v>
+      </c>
+      <c r="D151" s="3">
+        <v>5</v>
+      </c>
+      <c r="E151" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F151" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="G151" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="H151" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I151" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J151" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K151" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L151" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M151" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N151" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O151" s="3">
+        <v>0</v>
+      </c>
+      <c r="P151" s="3">
+        <v>15853081</v>
+      </c>
+      <c r="Q151" s="3">
+        <v>0</v>
+      </c>
+      <c r="R151" s="3">
+        <v>15853081</v>
+      </c>
+    </row>
+    <row r="152" outlineLevel="0" collapsed="0" hidden="0">
+      <c r="A152" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C152" s="3">
+        <v>5</v>
+      </c>
+      <c r="D152" s="3">
+        <v>5</v>
+      </c>
+      <c r="E152" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F152" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="G152" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="H152" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I152" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J152" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K152" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L152" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M152" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N152" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O152" s="3">
+        <v>0</v>
+      </c>
+      <c r="P152" s="3">
+        <v>47157460</v>
+      </c>
+      <c r="Q152" s="3">
+        <v>0</v>
+      </c>
+      <c r="R152" s="3">
+        <v>47157460</v>
+      </c>
+    </row>
+    <row r="153" outlineLevel="0" collapsed="0" hidden="0">
+      <c r="A153" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C153" s="3">
+        <v>5</v>
+      </c>
+      <c r="D153" s="3">
+        <v>5</v>
+      </c>
+      <c r="E153" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F153" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="G153" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="H153" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I153" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J153" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K153" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L153" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="M153" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N153" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O153" s="3">
+        <v>0</v>
+      </c>
+      <c r="P153" s="3">
+        <v>54606561</v>
+      </c>
+      <c r="Q153" s="3">
+        <v>0</v>
+      </c>
+      <c r="R153" s="3">
+        <v>54606561</v>
+      </c>
+    </row>
+    <row r="154" outlineLevel="0" collapsed="0" hidden="0">
+      <c r="A154" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C154" s="3">
+        <v>5</v>
+      </c>
+      <c r="D154" s="3">
+        <v>5</v>
+      </c>
+      <c r="E154" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="F154" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="G154" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="H154" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I154" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J154" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K154" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L154" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="M154" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N154" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="O154" s="3">
+        <v>0</v>
+      </c>
+      <c r="P154" s="3">
+        <v>65307008</v>
+      </c>
+      <c r="Q154" s="3">
+        <v>0</v>
+      </c>
+      <c r="R154" s="3">
+        <v>65307008</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M155" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="N155" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="O155" s="6">
         <v>7559544498</v>
       </c>
-      <c r="P148" s="6">
-        <v>7302435411</v>
-      </c>
-      <c r="Q148" s="6">
+      <c r="P155" s="6">
+        <v>7688339476</v>
+      </c>
+      <c r="Q155" s="6">
         <v>7290068461</v>
       </c>
-      <c r="R148" s="6">
-        <v>7571911448</v>
+      <c r="R155" s="6">
+        <v>7957815513</v>
       </c>
     </row>
   </sheetData>

</xml_diff>